<commit_message>
Atualiza lista de CADIFAs deferidas (nenhuma novidade em 16/09/2026)
Nenhuma linha nova por Nº CADIFA + Revisão. 10 linhas tiveram apenas a
Data Última Situação atualizada.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PNdTVVkDiotonib7AJhoo8
</commit_message>
<xml_diff>
--- a/cadifa_completo.xlsx
+++ b/cadifa_completo.xlsx
@@ -446,17 +446,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Sun Pharmaceutical Industries Limited</t>
+          <t>Xellia Pharmaceuticals Aps</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>cloridrato de sertralina</t>
+          <t>anfotericina b</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>25351114179202246</t>
+          <t>25351860617202322</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -466,24 +466,24 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Sun Pharmaceutical Industries Limited</t>
+          <t>Wanbury Limited</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>propionato de fluticasona</t>
+          <t>cloridrato de metformina</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>25351088020202421</t>
+          <t>25351454913202479</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -493,24 +493,24 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Dr Reddys Farmacêutica Do Brasil Ltda</t>
+          <t>Honour Lab Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>levetiracetam</t>
+          <t>empagliflozina</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>25351078614202423</t>
+          <t>25351427875202481</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -520,24 +520,24 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sun Pharmaceutical Industries Limited</t>
+          <t>Asolution Pharmaceuticals Pvt. Ltd.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>vismodegibe</t>
+          <t>sugamadex sódico</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>25351045971202677</t>
+          <t>25351793830202150</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -547,24 +547,24 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Shilpa Pharma Lifesciences Limited</t>
+          <t>Hetero Labs Limited</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>mesilato de lenvatinibe</t>
+          <t>cloridrato de atomoxetina</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>25351017275202590</t>
+          <t>25351114320202553</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -574,24 +574,24 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Hetero Labs Limited</t>
+          <t>Sun Pharmaceutical Industries Limited</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>cloridrato de atomoxetina</t>
+          <t>lacosamida</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>25351114320202553</t>
+          <t>25351226464202551</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -601,24 +601,24 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Asolution Pharmaceuticals Pvt. Ltd.</t>
+          <t>Harman Finochem Limited</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>sugamadex sódico</t>
+          <t>hemitartarato de norepinefrina monoidratada</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>25351793830202150</t>
+          <t>25351358693202453</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -628,24 +628,24 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>04/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Harman Finochem Limited</t>
+          <t>Synthon Bv</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>hemitartarato de norepinefrina monoidratada</t>
+          <t>lenalidomida</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>25351358693202453</t>
+          <t>25351807850202387</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -655,24 +655,24 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>02/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Synthon Bv</t>
+          <t>Sun Pharmaceutical Industries Limited</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>lenalidomida</t>
+          <t>dapagliflozina propanodiol monoidratado</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>25351807850202387</t>
+          <t>25351355090202408</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -682,24 +682,24 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>02/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Sun Pharmaceutical Industries Limited</t>
+          <t>Hetero Drugs Limited</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>lacosamida</t>
+          <t>mirtazapina</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>25351226464202551</t>
+          <t>25351268546202310</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -709,24 +709,24 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>02/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Wanbury Limited</t>
+          <t>Sun Pharmaceutical Industries Limited</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>cloridrato de metformina</t>
+          <t>cloridrato de sertralina</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>25351454913202479</t>
+          <t>25351114179202246</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -736,24 +736,24 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>02/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Honour Lab Limited</t>
+          <t>Sun Pharmaceutical Industries Limited</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>empagliflozina</t>
+          <t>propionato de fluticasona</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>25351427875202481</t>
+          <t>25351088020202421</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -763,24 +763,24 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>31/08/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Hetero Drugs Limited</t>
+          <t>Dr Reddys Farmacêutica Do Brasil Ltda</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>mirtazapina</t>
+          <t>levetiracetam</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>25351268546202310</t>
+          <t>25351078614202423</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>31/08/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
     </row>
@@ -802,12 +802,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>dapagliflozina propanodiol monoidratado</t>
+          <t>vismodegibe</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>25351355090202408</t>
+          <t>25351045971202677</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -817,24 +817,24 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>28/08/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Xellia Pharmaceuticals Aps</t>
+          <t>Shilpa Pharma Lifesciences Limited</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>anfotericina b</t>
+          <t>mesilato de lenvatinibe</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>25351860617202322</t>
+          <t>25351017275202590</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>28/08/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza lista de CADIFAs deferidas (execução automática)
1 CADIFA nova: Nº 25351145024202502, Revisão 001 (Heraeus Precious
Metals Gmbh & Co. Kg, cloridrato do ácido aminolevulínico), última
situação em 25/08/2026.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QiY6jYa65nRJgxqjXT3jJ7
</commit_message>
<xml_diff>
--- a/cadifa_completo.xlsx
+++ b/cadifa_completo.xlsx
@@ -932,7 +932,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Heraeus Deutschland Gmbh &amp; Co. Kg</t>
+          <t>Heraeus Precious Metals Gmbh &amp; Co. Kg</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>001.1</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza CADIFAs deferidas (682 linhas, 4 novas)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FFD6pLziFw1etd47HGpi3T
</commit_message>
<xml_diff>
--- a/cadifa_completo.xlsx
+++ b/cadifa_completo.xlsx
@@ -2810,7 +2810,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>001.1</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -3323,7 +3323,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>001.1</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -3620,7 +3620,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>001.1</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -17849,7 +17849,7 @@
       </c>
       <c r="D646" t="inlineStr">
         <is>
-          <t>005</t>
+          <t>005.1</t>
         </is>
       </c>
       <c r="E646" t="inlineStr">

</xml_diff>